<commit_message>
feat(data): iş ilanları veri setini zenginleştir
- 200 -> 247 ilan. 22 hedef rolün tamamında en az birkaç örnek
  olacak şekilde zayıf/sıfır kategoriler dolduruldu
  (digital_marketing_specialist 0->7, graphic_designer, hr_specialist,
  database_administrator, backend_developer, devops_engineer,
  systems_administrator, data_scientist ve diğerleri)
- 3 satırdaki eksik job_domain düzeltildi, tekrar eden id / boş
  açıklama kontrolü yapıldı (temiz çıktı)
- test: backend/devops/data-scientist örnek CV'lerinde en iyi
  eşleşmeler %94-98 aralığında, tamamı alakalı başlıklarla dönüyor
</commit_message>
<xml_diff>
--- a/backend/data/jobs_dataset.xlsx
+++ b/backend/data/jobs_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O201"/>
+  <dimension ref="A1:O248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,9 +538,6 @@
       </c>
       <c r="I2" t="n">
         <v>5656</v>
-      </c>
-      <c r="J2" t="n">
-        <v/>
       </c>
       <c r="K2" t="b">
         <v>0</v>
@@ -987,9 +984,6 @@
       </c>
       <c r="I8" t="n">
         <v>1182</v>
-      </c>
-      <c r="J8" t="n">
-        <v/>
       </c>
       <c r="K8" t="b">
         <v>1</v>
@@ -1284,9 +1278,6 @@
       <c r="I12" t="n">
         <v>1038</v>
       </c>
-      <c r="J12" t="n">
-        <v/>
-      </c>
       <c r="K12" t="b">
         <v>1</v>
       </c>
@@ -1861,9 +1852,6 @@
       </c>
       <c r="I20" t="n">
         <v>945</v>
-      </c>
-      <c r="J20" t="n">
-        <v/>
       </c>
       <c r="K20" t="b">
         <v>1</v>
@@ -2372,9 +2360,6 @@
       </c>
       <c r="I27" t="n">
         <v>812</v>
-      </c>
-      <c r="J27" t="n">
-        <v/>
       </c>
       <c r="K27" t="b">
         <v>1</v>
@@ -2829,9 +2814,6 @@
       <c r="I33" t="n">
         <v>655</v>
       </c>
-      <c r="J33" t="n">
-        <v/>
-      </c>
       <c r="K33" t="b">
         <v>0</v>
       </c>
@@ -2958,9 +2940,6 @@
       </c>
       <c r="I35" t="n">
         <v>620</v>
-      </c>
-      <c r="J35" t="n">
-        <v/>
       </c>
       <c r="K35" t="b">
         <v>0</v>
@@ -3226,9 +3205,6 @@
       </c>
       <c r="I39" t="n">
         <v>561</v>
-      </c>
-      <c r="J39" t="n">
-        <v/>
       </c>
       <c r="K39" t="b">
         <v>1</v>
@@ -4295,9 +4271,6 @@
       <c r="I54" t="n">
         <v>479</v>
       </c>
-      <c r="J54" t="n">
-        <v/>
-      </c>
       <c r="K54" t="b">
         <v>0</v>
       </c>
@@ -4656,9 +4629,6 @@
       <c r="I59" t="n">
         <v>462</v>
       </c>
-      <c r="J59" t="n">
-        <v/>
-      </c>
       <c r="K59" t="b">
         <v>0</v>
       </c>
@@ -4791,9 +4761,6 @@
       </c>
       <c r="I61" t="n">
         <v>455</v>
-      </c>
-      <c r="J61" t="n">
-        <v/>
       </c>
       <c r="K61" t="b">
         <v>1</v>
@@ -5721,9 +5688,6 @@
       <c r="I74" t="n">
         <v>381</v>
       </c>
-      <c r="J74" t="n">
-        <v/>
-      </c>
       <c r="K74" t="b">
         <v>1</v>
       </c>
@@ -6519,9 +6483,6 @@
       <c r="I85" t="n">
         <v>348</v>
       </c>
-      <c r="J85" t="n">
-        <v/>
-      </c>
       <c r="K85" t="b">
         <v>0</v>
       </c>
@@ -6924,9 +6885,6 @@
       <c r="I91" t="n">
         <v>337</v>
       </c>
-      <c r="J91" t="n">
-        <v/>
-      </c>
       <c r="K91" t="b">
         <v>0</v>
       </c>
@@ -7410,9 +7368,6 @@
       <c r="I98" t="n">
         <v>325</v>
       </c>
-      <c r="J98" t="n">
-        <v/>
-      </c>
       <c r="K98" t="b">
         <v>0</v>
       </c>
@@ -7485,9 +7440,6 @@
       </c>
       <c r="I99" t="n">
         <v>323</v>
-      </c>
-      <c r="J99" t="n">
-        <v/>
       </c>
       <c r="K99" t="b">
         <v>1</v>
@@ -7564,9 +7516,6 @@
       <c r="I100" t="n">
         <v>323</v>
       </c>
-      <c r="J100" t="n">
-        <v/>
-      </c>
       <c r="K100" t="b">
         <v>1</v>
       </c>
@@ -8133,9 +8082,6 @@
       </c>
       <c r="I108" t="n">
         <v>300</v>
-      </c>
-      <c r="J108" t="n">
-        <v/>
       </c>
       <c r="K108" t="b">
         <v>0</v>
@@ -8888,9 +8834,6 @@
       <c r="I119" t="n">
         <v>285</v>
       </c>
-      <c r="J119" t="n">
-        <v/>
-      </c>
       <c r="K119" t="b">
         <v>1</v>
       </c>
@@ -8899,8 +8842,10 @@
           <t xml:space="preserve">$80,000.00 </t>
         </is>
       </c>
-      <c r="M119" t="n">
-        <v/>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
       </c>
       <c r="N119" t="n">
         <v>1342014</v>
@@ -9236,9 +9181,6 @@
       <c r="I124" t="n">
         <v>283</v>
       </c>
-      <c r="J124" t="n">
-        <v/>
-      </c>
       <c r="K124" t="b">
         <v>1</v>
       </c>
@@ -9443,9 +9385,6 @@
       <c r="I127" t="n">
         <v>280</v>
       </c>
-      <c r="J127" t="n">
-        <v/>
-      </c>
       <c r="K127" t="b">
         <v>1</v>
       </c>
@@ -9454,8 +9393,10 @@
           <t xml:space="preserve">$125,000.00 </t>
         </is>
       </c>
-      <c r="M127" t="n">
-        <v/>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
       </c>
       <c r="N127" t="n">
         <v>75752648</v>
@@ -9813,9 +9754,6 @@
       <c r="I132" t="n">
         <v>274</v>
       </c>
-      <c r="J132" t="n">
-        <v/>
-      </c>
       <c r="K132" t="b">
         <v>0</v>
       </c>
@@ -9966,9 +9904,6 @@
       <c r="I134" t="n">
         <v>273</v>
       </c>
-      <c r="J134" t="n">
-        <v/>
-      </c>
       <c r="K134" t="b">
         <v>0</v>
       </c>
@@ -10101,9 +10036,6 @@
       <c r="I136" t="n">
         <v>271</v>
       </c>
-      <c r="J136" t="n">
-        <v/>
-      </c>
       <c r="K136" t="b">
         <v>1</v>
       </c>
@@ -10112,8 +10044,10 @@
           <t xml:space="preserve">$195,000.00 </t>
         </is>
       </c>
-      <c r="M136" t="n">
-        <v/>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
       </c>
       <c r="N136" t="n">
         <v>49122753</v>
@@ -10923,9 +10857,6 @@
       <c r="I148" t="n">
         <v>247</v>
       </c>
-      <c r="J148" t="n">
-        <v/>
-      </c>
       <c r="K148" t="b">
         <v>0</v>
       </c>
@@ -11129,9 +11060,6 @@
       </c>
       <c r="I151" t="n">
         <v>240</v>
-      </c>
-      <c r="J151" t="n">
-        <v/>
       </c>
       <c r="K151" t="b">
         <v>0</v>
@@ -11337,9 +11265,6 @@
       <c r="I154" t="n">
         <v>237</v>
       </c>
-      <c r="J154" t="n">
-        <v/>
-      </c>
       <c r="K154" t="b">
         <v>1</v>
       </c>
@@ -11470,9 +11395,6 @@
       </c>
       <c r="I156" t="n">
         <v>236</v>
-      </c>
-      <c r="J156" t="n">
-        <v/>
       </c>
       <c r="K156" t="b">
         <v>0</v>
@@ -11704,9 +11626,6 @@
       <c r="I159" t="n">
         <v>232</v>
       </c>
-      <c r="J159" t="n">
-        <v/>
-      </c>
       <c r="K159" t="b">
         <v>1</v>
       </c>
@@ -12030,9 +11949,6 @@
       </c>
       <c r="I164" t="n">
         <v>228</v>
-      </c>
-      <c r="J164" t="n">
-        <v/>
       </c>
       <c r="K164" t="b">
         <v>0</v>
@@ -13204,9 +13120,6 @@
       <c r="I180" t="n">
         <v>211</v>
       </c>
-      <c r="J180" t="n">
-        <v/>
-      </c>
       <c r="K180" t="b">
         <v>1</v>
       </c>
@@ -13399,9 +13312,6 @@
       </c>
       <c r="I183" t="n">
         <v>209</v>
-      </c>
-      <c r="J183" t="n">
-        <v/>
       </c>
       <c r="K183" t="b">
         <v>0</v>
@@ -14707,6 +14617,2967 @@
         <v>1</v>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>9000000001</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Digital Marketing Specialist</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Northwind Retail Co. is hiring a Digital Marketing Specialist to own paid and organic acquisition channels for our e-commerce brand. You will plan and execute campaigns across Google Ads, Meta Ads, and email, and report on CAC, ROAS, and conversion funnels. What You'll Do: Manage monthly paid media budget across search and social; build and optimize landing pages with A/B testing; own the email and SMS marketing calendar in Klaviyo; track campaign performance in Google Analytics 4 and build weekly dashboards; coordinate with the design team on creative assets. What We Look For: 2-4 years of hands-on digital marketing experience; proficiency with Google Ads, Meta Ads Manager, and GA4; working knowledge of SEO fundamentals and keyword research tools (SEMrush or Ahrefs); strong analytical skills and comfort with spreadsheets; excellent written communication for ad copy and email content.</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="G202" t="n">
+        <v>669</v>
+      </c>
+      <c r="H202" t="b">
+        <v>1</v>
+      </c>
+      <c r="I202" t="n">
+        <v>1112</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K202" t="b">
+        <v>1</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$72,000.00 </t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="N202" t="n">
+        <v>89903925</v>
+      </c>
+      <c r="O202" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>9000000002</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>SEO &amp; Content Marketing Specialist</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Brightpath Media is looking for an SEO &amp; Content Marketing Specialist to grow organic traffic for our portfolio of client websites. You'll drive keyword research, on-page optimization, and a content calendar that turns into ranking pages. Responsibilities: conduct technical SEO audits and fix crawlability/indexing issues; build keyword clusters and briefs for writers; manage backlink outreach and internal linking strategy; monitor rankings and organic traffic in Google Search Console and SEMrush; collaborate with content writers and designers on blog and landing page production. Requirements: 1-3 years in SEO or content marketing; familiarity with Google Search Console, SEMrush or Ahrefs, and basic HTML; strong writing and editing skills; data-driven mindset with monthly reporting experience.</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G203" t="n">
+        <v>296</v>
+      </c>
+      <c r="H203" t="b">
+        <v>1</v>
+      </c>
+      <c r="I203" t="n">
+        <v>2206</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K203" t="b">
+        <v>1</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$65,000.00 </t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="N203" t="n">
+        <v>89903926</v>
+      </c>
+      <c r="O203" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>9000000003</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Performance Marketing Manager</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Loopline Commerce is seeking a Performance Marketing Manager to lead paid acquisition strategy across search, social, and programmatic channels for a fast-growing D2C brand. What You'll Do: own the full-funnel paid media budget and scale profitable campaigns on Google Ads, Meta, and TikTok Ads; run continuous A/B tests on creative and bidding strategy; partner with analytics on attribution modeling and incrementality testing; manage relationships with external media agencies; present growth results to leadership. What We're Looking For: 4+ years in performance/digital marketing with budgets over $500K/year; strong command of Google Ads, Meta Ads Manager, and marketing analytics platforms; experience with attribution and LTV/CAC modeling; excellent stakeholder communication.</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="G204" t="n">
+        <v>769</v>
+      </c>
+      <c r="H204" t="b">
+        <v>0</v>
+      </c>
+      <c r="I204" t="n">
+        <v>1039</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K204" t="b">
+        <v>0</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$95,000.00 </t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="N204" t="n">
+        <v>89903927</v>
+      </c>
+      <c r="O204" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>9000000004</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Growth Marketing Specialist</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Nova Consumer Group is hiring a Social Media &amp; Growth Marketing Specialist to grow our brand presence on Instagram, TikTok, and YouTube Shorts. Responsibilities: plan and publish a weekly content calendar across social platforms; run influencer and UGC collaborations; track engagement, follower growth, and click-through rate; test short-form video hooks and captions to improve reach; support paid social boosting of top-performing organic posts. Requirements: 0-2 years of experience in social media or growth marketing (internships count); native understanding of TikTok/Instagram trends and short-form video editing tools (CapCut or similar); basic familiarity with Meta Ads Manager; strong copywriting instincts.</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G205" t="n">
+        <v>573</v>
+      </c>
+      <c r="H205" t="b">
+        <v>1</v>
+      </c>
+      <c r="I205" t="n">
+        <v>912</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K205" t="b">
+        <v>0</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$55,000.00 </t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="N205" t="n">
+        <v>89903928</v>
+      </c>
+      <c r="O205" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>9000000005</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Email Marketing &amp; CRM Specialist</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Harborview Retail is looking for an Email Marketing &amp; CRM Specialist to own lifecycle campaigns that drive repeat purchases across our customer base. What You'll Do: build and segment email flows (welcome, abandoned cart, win-back) in Klaviyo; run A/B tests on subject lines, send times, and content blocks; maintain customer segmentation and CRM hygiene; monitor deliverability, open rate, and revenue-per-email; collaborate with design on email templates. What We Look For: 2+ years running email/CRM campaigns, ideally with Klaviyo or HubSpot; strong grasp of segmentation and lifecycle marketing concepts; comfortable with basic HTML for email templates; analytical mindset with weekly reporting habit.</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G206" t="n">
+        <v>47</v>
+      </c>
+      <c r="H206" t="b">
+        <v>1</v>
+      </c>
+      <c r="I206" t="n">
+        <v>444</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K206" t="b">
+        <v>1</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$68,000.00 </t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="N206" t="n">
+        <v>89903929</v>
+      </c>
+      <c r="O206" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>9000000006</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Graphic Designer</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Studio Kestrel is hiring a Graphic Designer to create visual assets across digital and print for a range of consumer brand clients. Responsibilities: design social media graphics, email templates, and paid ad creative in Figma and Adobe Illustrator; maintain and extend brand style guides across multiple client accounts; prepare print-ready files for packaging and event collateral; collaborate with marketing and content teams on campaign concepts; present design work to clients and incorporate feedback. Requirements: 3+ years of graphic design experience with a strong portfolio; expert in Adobe Creative Suite (Illustrator, Photoshop, InDesign) and Figma; solid understanding of typography, color theory, and layout; ability to manage multiple projects under deadline.</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="G207" t="n">
+        <v>253</v>
+      </c>
+      <c r="H207" t="b">
+        <v>1</v>
+      </c>
+      <c r="I207" t="n">
+        <v>4339</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K207" t="b">
+        <v>0</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$70,000.00 </t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="N207" t="n">
+        <v>89903930</v>
+      </c>
+      <c r="O207" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>9000000007</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Brand &amp; Visual Designer</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Anvil Creative Agency is seeking a Brand &amp; Visual Designer to shape brand identity systems for startup clients. What You'll Do: design logos, brand guidelines, and marketing collateral from concept to final delivery; build presentation decks and pitch materials in Figma; iterate on visual concepts based on client feedback in fast turnaround cycles; support web and landing page design with UI mockups. What We Look For: 2-4 years in brand or visual design; strong portfolio showing logo and identity work; proficiency in Figma, Illustrator, and Photoshop; excellent visual storytelling and attention to detail.</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G208" t="n">
+        <v>589</v>
+      </c>
+      <c r="H208" t="b">
+        <v>1</v>
+      </c>
+      <c r="I208" t="n">
+        <v>1828</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K208" t="b">
+        <v>0</v>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$62,000.00 </t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="N208" t="n">
+        <v>89903931</v>
+      </c>
+      <c r="O208" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>9000000008</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Junior Graphic Designer</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Lumen Print &amp; Design is looking for a Junior Graphic Designer to support our creative team on a variety of print and digital projects. Responsibilities: produce flyers, brochures, and packaging mockups under senior designer direction; prepare files for print production (bleed, color profiles, resolution checks); assist with resizing and adapting creative assets for different formats and platforms; organize and maintain the design asset library. Requirements: 0-1 years of professional design experience or a strong design school portfolio; working knowledge of Adobe Illustrator and Photoshop; basic understanding of print production requirements; eagerness to learn and take feedback.</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="G209" t="n">
+        <v>733</v>
+      </c>
+      <c r="H209" t="b">
+        <v>0</v>
+      </c>
+      <c r="I209" t="n">
+        <v>4664</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K209" t="b">
+        <v>0</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$48,000.00 </t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="N209" t="n">
+        <v>89903932</v>
+      </c>
+      <c r="O209" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>9000000009</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Senior Graphic Designer, Marketing</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Northwind Retail Co. is hiring a Senior Graphic Designer to lead visual design for our marketing team. What You'll Do: own the visual direction for seasonal campaigns across web, email, and social; mentor junior designers and review their work; partner closely with copywriters and the performance marketing team on ad creative that converts; manage the brand system and ensure consistency across all customer touchpoints. What We're Looking For: 5+ years of graphic design experience, ideally in retail or e-commerce; expert-level Figma and Adobe Creative Suite skills; strong portfolio demonstrating campaign-level creative work; experience giving and receiving design critique.</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>474</v>
+      </c>
+      <c r="H210" t="b">
+        <v>1</v>
+      </c>
+      <c r="I210" t="n">
+        <v>5027</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K210" t="b">
+        <v>0</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$88,000.00 </t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="N210" t="n">
+        <v>89903925</v>
+      </c>
+      <c r="O210" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>9000000010</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>HR Specialist</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Meridian Group is hiring an HR Specialist to support day-to-day people operations for a 200-person organization. Responsibilities: manage onboarding and offboarding paperwork and orientation sessions; maintain employee records and HRIS data accuracy; support benefits enrollment and answer employee questions; assist with policy communication and compliance documentation; coordinate performance review cycles with managers. Requirements: 2+ years in an HR generalist or HR specialist role; familiarity with an HRIS platform (Workday, BambooHR, or similar); strong organizational skills and attention to detail; discretion when handling confidential employee information.</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Dallas, TX</t>
+        </is>
+      </c>
+      <c r="G211" t="n">
+        <v>21</v>
+      </c>
+      <c r="H211" t="b">
+        <v>0</v>
+      </c>
+      <c r="I211" t="n">
+        <v>1507</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K211" t="b">
+        <v>0</v>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$60,000.00 </t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="N211" t="n">
+        <v>89903933</v>
+      </c>
+      <c r="O211" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>9000000011</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Human Resources Generalist</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Cobalt Manufacturing is looking for a Human Resources Generalist to own HR operations across our two facilities. What You'll Do: manage full-cycle recruiting for hourly and salaried roles; administer benefits, leave of absence, and workers' compensation cases; advise managers on performance issues and progressive discipline; ensure compliance with state and federal employment law; run new-hire orientation and safety onboarding. What We Look For: 3-5 years of HR generalist experience, ideally in a manufacturing or industrial setting; solid knowledge of employment law and HR compliance; experience with an HRIS and applicant tracking system; strong interpersonal and conflict-resolution skills.</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ</t>
+        </is>
+      </c>
+      <c r="G212" t="n">
+        <v>363</v>
+      </c>
+      <c r="H212" t="b">
+        <v>0</v>
+      </c>
+      <c r="I212" t="n">
+        <v>2476</v>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K212" t="b">
+        <v>1</v>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$72,000.00 </t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="N212" t="n">
+        <v>89903934</v>
+      </c>
+      <c r="O212" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>9000000012</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Talent Acquisition Specialist</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Brightpath Media is hiring a Talent Acquisition Specialist to manage recruiting for our growing marketing and creative teams. Responsibilities: source and screen candidates using LinkedIn Recruiter and our applicant tracking system; coordinate interview loops and collect structured feedback from hiring panels; manage offer negotiation and background check processes; build a pipeline of passive candidates for hard-to-fill creative roles; track recruiting metrics like time-to-fill and source of hire. Requirements: 2+ years of full-cycle recruiting experience; hands-on experience with an ATS (Greenhouse, Lever, or similar) and LinkedIn Recruiter; excellent communication and candidate relationship management skills.</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G213" t="n">
+        <v>796</v>
+      </c>
+      <c r="H213" t="b">
+        <v>1</v>
+      </c>
+      <c r="I213" t="n">
+        <v>2957</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K213" t="b">
+        <v>1</v>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$66,000.00 </t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="N213" t="n">
+        <v>89903926</v>
+      </c>
+      <c r="O213" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>9000000013</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>HR Business Partner</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Anchorline Logistics is seeking an HR Business Partner to support our operations leadership team. What You'll Do: partner with department heads on workforce planning, org design, and performance management; coach managers through employee relations issues and disciplinary processes; analyze headcount and attrition data to inform retention strategy; lead compensation review cycles in partnership with the People Analytics team; champion engagement initiatives across a distributed warehouse workforce. What We're Looking For: 5+ years as an HR generalist or HRBP, ideally supporting operations or logistics teams; strong grounding in employment law and progressive discipline practices; comfortable working with HR data and building manager-facing reports.</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="G214" t="n">
+        <v>404</v>
+      </c>
+      <c r="H214" t="b">
+        <v>0</v>
+      </c>
+      <c r="I214" t="n">
+        <v>992</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K214" t="b">
+        <v>0</v>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$98,000.00 </t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="N214" t="n">
+        <v>89903935</v>
+      </c>
+      <c r="O214" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>9000000014</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Database Administrator</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Ledger Financial Systems is hiring a Database Administrator to maintain and optimize our production database fleet supporting transaction processing. Responsibilities: administer and tune PostgreSQL and SQL Server instances for performance and reliability; design backup, replication, and disaster recovery procedures; monitor query performance and resolve slow-running queries with indexing and execution plan analysis; manage database security, access control, and encryption at rest; support schema migrations for engineering teams. Requirements: 4+ years as a DBA managing production relational databases; strong SQL tuning and indexing skills; experience with backup/recovery tooling and high-availability replication setups; familiarity with monitoring tools such as pgAdmin, Datadog, or similar.</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Charlotte, NC</t>
+        </is>
+      </c>
+      <c r="G215" t="n">
+        <v>367</v>
+      </c>
+      <c r="H215" t="b">
+        <v>0</v>
+      </c>
+      <c r="I215" t="n">
+        <v>5145</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K215" t="b">
+        <v>0</v>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$105,000.00 </t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N215" t="n">
+        <v>89903936</v>
+      </c>
+      <c r="O215" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>9000000015</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>PostgreSQL Database Administrator</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Vertex Cloud Solutions is looking for a PostgreSQL Database Administrator to support our multi-tenant SaaS platform. What You'll Do: manage PostgreSQL clusters across staging and production, including partitioning and vacuum strategy for large tables; automate routine DBA tasks with scripts and infrastructure-as-code; participate in an on-call rotation for database incidents; collaborate with backend engineers on schema design and query optimization; evaluate and roll out extensions like pgvector and pg_stat_statements. Requirements: 3+ years of hands-on PostgreSQL administration; solid understanding of replication, connection pooling (PgBouncer), and partitioning; comfortable with Linux command line and basic scripting (Bash or Python); experience working in cloud environments (AWS RDS or self-managed).</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G216" t="n">
+        <v>59</v>
+      </c>
+      <c r="H216" t="b">
+        <v>1</v>
+      </c>
+      <c r="I216" t="n">
+        <v>3963</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K216" t="b">
+        <v>0</v>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$110,000.00 </t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N216" t="n">
+        <v>89903937</v>
+      </c>
+      <c r="O216" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>9000000016</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Junior Database Administrator</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Harborview Retail is hiring a Junior Database Administrator to support our IT operations team. Responsibilities: assist senior DBAs with routine maintenance tasks like backups, index rebuilds, and patching; monitor database health dashboards and escalate anomalies; help troubleshoot slow queries reported by application teams; document database configurations and runbooks; support user access requests and permission changes. Requirements: 0-2 years of database administration or strong academic/lab experience with SQL Server or MySQL; understanding of basic SQL, indexing, and normalization concepts; eagerness to learn production database operations.</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Columbus, OH</t>
+        </is>
+      </c>
+      <c r="G217" t="n">
+        <v>402</v>
+      </c>
+      <c r="H217" t="b">
+        <v>0</v>
+      </c>
+      <c r="I217" t="n">
+        <v>845</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K217" t="b">
+        <v>0</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$62,000.00 </t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N217" t="n">
+        <v>89903929</v>
+      </c>
+      <c r="O217" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>9000000017</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Senior DBA, Data Platform</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Ledger Financial Systems is seeking a Senior DBA to own the reliability of our core data platform. What You'll Do: lead capacity planning and scaling strategy across a fleet of PostgreSQL and MySQL instances; drive standards for backup verification and disaster recovery testing; mentor junior DBAs and review schema change proposals; partner with the security team on audit and compliance requirements (SOC 2); own incident postmortems for database-related outages. What We're Looking For: 6+ years of production DBA experience in a regulated or high-availability environment; deep expertise in query tuning, replication topologies, and backup/recovery; strong communication skills for cross-team collaboration.</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+      <c r="G218" t="n">
+        <v>864</v>
+      </c>
+      <c r="H218" t="b">
+        <v>1</v>
+      </c>
+      <c r="I218" t="n">
+        <v>5349</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K218" t="b">
+        <v>0</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$125,000.00 </t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N218" t="n">
+        <v>89903936</v>
+      </c>
+      <c r="O218" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>9000000018</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Backend Developer (Python/FastAPI)</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Vertex Cloud Solutions is hiring a Backend Developer to build and scale the API layer of our SaaS platform. Responsibilities: design and implement RESTful APIs using Python and FastAPI; model and optimize PostgreSQL schemas with SQLAlchemy; add caching and background job processing with Redis and Celery; write unit and integration tests to keep the codebase reliable as we scale; containerize services with Docker and support CI/CD pipelines. Requirements: 3+ years of backend development experience in Python; hands-on experience with FastAPI or Django REST Framework; solid understanding of relational database design and SQL performance; familiarity with Docker and basic CI/CD concepts; comfortable working in an agile, fast-iterating team.</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G219" t="n">
+        <v>897</v>
+      </c>
+      <c r="H219" t="b">
+        <v>1</v>
+      </c>
+      <c r="I219" t="n">
+        <v>3162</v>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K219" t="b">
+        <v>0</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$115,000.00 </t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N219" t="n">
+        <v>89903937</v>
+      </c>
+      <c r="O219" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>9000000019</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Backend Software Engineer</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Loopline Commerce is looking for a Backend Software Engineer to own core services powering our checkout and order management systems. What You'll Do: design and maintain microservices in Python and Go; build event-driven pipelines with Kafka for order and inventory events; ensure high availability and observability with structured logging and tracing; participate in system design reviews and on-call rotation; optimize PostgreSQL queries under high transaction volume. What We're Looking For: 4+ years of backend engineering experience; strong grasp of microservice architecture and API design; experience with message queues (Kafka, RabbitMQ, or SQS); solid SQL and database performance skills; comfortable operating production systems at scale.</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="G220" t="n">
+        <v>736</v>
+      </c>
+      <c r="H220" t="b">
+        <v>1</v>
+      </c>
+      <c r="I220" t="n">
+        <v>769</v>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K220" t="b">
+        <v>1</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$135,000.00 </t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N220" t="n">
+        <v>89903927</v>
+      </c>
+      <c r="O220" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>9000000020</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Junior Backend Developer</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Nova Consumer Group is hiring a Junior Backend Developer to join our engineering team building internal tools and customer-facing APIs. Responsibilities: implement API endpoints and business logic under senior engineer guidance using Python and Flask; write unit tests and participate in code review; fix bugs and small feature requests from the product backlog; learn our data model and contribute to database migrations. Requirements: 0-2 years of backend development experience (internships and bootcamp projects count); working knowledge of Python and SQL; understanding of REST API basics and Git version control; strong eagerness to learn from senior teammates.</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="G221" t="n">
+        <v>248</v>
+      </c>
+      <c r="H221" t="b">
+        <v>0</v>
+      </c>
+      <c r="I221" t="n">
+        <v>2570</v>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K221" t="b">
+        <v>0</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$70,000.00 </t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N221" t="n">
+        <v>89903928</v>
+      </c>
+      <c r="O221" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>9000000021</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Senior Backend Engineer, Payments</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Ledger Financial Systems is seeking a Senior Backend Engineer to build the services that process customer payments and settlements. What You'll Do: design idempotent, auditable payment processing services in Java and Python; enforce strict data consistency using PostgreSQL transactions and distributed locking; lead technical design reviews for new payment features; mentor mid-level engineers on API design and testing practices; work closely with compliance on PCI-DSS requirements. What We're Looking For: 6+ years of backend engineering experience, ideally in fintech or payments; deep understanding of transactional database design and concurrency; experience with high-reliability, audit-heavy systems; strong communication and mentorship skills.</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="G222" t="n">
+        <v>890</v>
+      </c>
+      <c r="H222" t="b">
+        <v>0</v>
+      </c>
+      <c r="I222" t="n">
+        <v>2107</v>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K222" t="b">
+        <v>0</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$155,000.00 </t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N222" t="n">
+        <v>89903936</v>
+      </c>
+      <c r="O222" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>9000000022</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Backend Engineer, Internal Tools</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Anchorline Logistics needs a contract Backend Engineer to build internal tooling for our warehouse operations team. Responsibilities: build internal APIs in Node.js and Express that integrate with our warehouse management system; design PostgreSQL schemas for shipment tracking and inventory reconciliation; build simple admin dashboards backed by these APIs; write clear documentation for the ops team who will maintain the tools. Requirements: 3+ years of backend development experience with Node.js or Python; comfortable working independently on a 3-month contract; solid SQL and API design skills; prior experience building internal/admin tooling is a plus.</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>HOURLY</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G223" t="n">
+        <v>404</v>
+      </c>
+      <c r="H223" t="b">
+        <v>1</v>
+      </c>
+      <c r="I223" t="n">
+        <v>2477</v>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K223" t="b">
+        <v>0</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$75.00 </t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N223" t="n">
+        <v>89903938</v>
+      </c>
+      <c r="O223" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>9000000023</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Backend Developer, API Platform</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Harborview Retail is hiring a Backend Developer to join our API platform team responsible for the public developer API. What You'll Do: implement and version REST endpoints consumed by external partners; maintain API documentation with OpenAPI/Swagger; add rate limiting, authentication, and usage analytics for API consumers; work with QA on contract and integration testing. What We Look For: 2+ years of backend development experience with Python or Node.js; understanding of REST API design principles and versioning strategies; familiarity with OAuth2/JWT authentication; strong written communication for developer-facing documentation.</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="G224" t="n">
+        <v>869</v>
+      </c>
+      <c r="H224" t="b">
+        <v>1</v>
+      </c>
+      <c r="I224" t="n">
+        <v>3188</v>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K224" t="b">
+        <v>1</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$92,000.00 </t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N224" t="n">
+        <v>89903929</v>
+      </c>
+      <c r="O224" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>9000000024</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Vertex Cloud Solutions is hiring a DevOps Engineer to own our CI/CD pipelines and cloud infrastructure. Responsibilities: build and maintain Terraform modules for AWS infrastructure; design and improve GitHub Actions pipelines for build, test, and deploy; manage Kubernetes clusters running our microservices; set up monitoring and alerting with Prometheus and Grafana; support incident response and postmortems. Requirements: 3+ years of DevOps or infrastructure engineering experience; hands-on Terraform and AWS (EC2, EKS, RDS, S3) experience; solid Docker and Kubernetes skills; scripting ability in Python or Bash; on-call experience for production systems.</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G225" t="n">
+        <v>378</v>
+      </c>
+      <c r="H225" t="b">
+        <v>1</v>
+      </c>
+      <c r="I225" t="n">
+        <v>1916</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K225" t="b">
+        <v>0</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$120,000.00 </t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N225" t="n">
+        <v>89903937</v>
+      </c>
+      <c r="O225" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>9000000025</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Site Reliability Engineer</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Ledger Financial Systems is looking for a Site Reliability Engineer to keep our transaction platform highly available. What You'll Do: define and track SLOs/SLIs across core services; build automated remediation for common incident patterns; run chaos engineering exercises to validate failover paths; improve observability with distributed tracing and structured logging; participate in a 24/7 on-call rotation with a healthy escalation process. What We're Looking For: 4+ years in SRE, DevOps, or production engineering; strong Kubernetes and cloud infrastructure experience (AWS or GCP); comfortable writing automation in Python or Go; experience with incident management and postmortem culture.</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="G226" t="n">
+        <v>733</v>
+      </c>
+      <c r="H226" t="b">
+        <v>1</v>
+      </c>
+      <c r="I226" t="n">
+        <v>5799</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K226" t="b">
+        <v>0</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$140,000.00 </t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N226" t="n">
+        <v>89903936</v>
+      </c>
+      <c r="O226" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>9000000026</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Cloud DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Anchorline Logistics is hiring a Cloud DevOps Engineer to modernize our infrastructure as we migrate from on-prem to AWS. Responsibilities: write Terraform and Ansible to automate infrastructure provisioning; containerize legacy applications with Docker; build CI/CD pipelines in GitLab CI for gradual migration of services; monitor cost and performance of cloud resources; document migration runbooks for the engineering team. Requirements: 2+ years of DevOps or cloud infrastructure experience; working knowledge of Terraform and AWS; experience with Docker and at least one CI/CD platform; comfortable with Linux administration and shell scripting.</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="G227" t="n">
+        <v>638</v>
+      </c>
+      <c r="H227" t="b">
+        <v>1</v>
+      </c>
+      <c r="I227" t="n">
+        <v>5401</v>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K227" t="b">
+        <v>1</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$98,000.00 </t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N227" t="n">
+        <v>89903935</v>
+      </c>
+      <c r="O227" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>9000000027</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>DevOps Engineer, Platform Team</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Loopline Commerce is seeking a DevOps Engineer for our platform team supporting checkout and inventory services. What You'll Do: manage Kubernetes deployments across staging and production; build self-service tooling so product teams can deploy safely without DevOps bottlenecks; own secrets management and access control across cloud environments; automate capacity scaling based on traffic patterns during peak shopping events. What We Look For: 3+ years of DevOps experience in a high-traffic e-commerce or SaaS environment; strong Kubernetes and Helm skills; experience with GitOps workflows (ArgoCD or Flux); solid understanding of networking and security fundamentals in cloud environments.</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>761</v>
+      </c>
+      <c r="H228" t="b">
+        <v>1</v>
+      </c>
+      <c r="I228" t="n">
+        <v>2205</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K228" t="b">
+        <v>1</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$125,000.00 </t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N228" t="n">
+        <v>89903927</v>
+      </c>
+      <c r="O228" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>9000000028</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Junior DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Nova Consumer Group is hiring a Junior DevOps Engineer to support our infrastructure team. Responsibilities: help maintain CI/CD pipelines and fix build failures; assist with Docker image builds and basic Kubernetes deployments under senior guidance; monitor dashboards and escalate anomalies to senior engineers; write and improve internal documentation for deployment processes. Requirements: 0-2 years of DevOps, sysadmin, or infrastructure experience; basic familiarity with Linux, Docker, and Git; willingness to learn Terraform and cloud platforms (AWS or GCP) on the job.</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>403</v>
+      </c>
+      <c r="H229" t="b">
+        <v>0</v>
+      </c>
+      <c r="I229" t="n">
+        <v>2411</v>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K229" t="b">
+        <v>0</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$75,000.00 </t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N229" t="n">
+        <v>89903928</v>
+      </c>
+      <c r="O229" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>9000000029</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>DevOps Engineer, CI/CD</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Brightpath Media needs a contract DevOps Engineer to modernize our build and release pipelines over a 4-month engagement. Responsibilities: migrate Jenkins pipelines to GitHub Actions; containerize remaining legacy services; set up automated staging environments for QA; document the new deployment process for the internal team to maintain afterward. Requirements: 3+ years of CI/CD and DevOps experience; hands-on GitHub Actions and Docker experience; prior experience migrating from Jenkins is a strong plus; comfortable working independently on a fixed-scope contract.</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>HOURLY</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>670</v>
+      </c>
+      <c r="H230" t="b">
+        <v>1</v>
+      </c>
+      <c r="I230" t="n">
+        <v>5837</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K230" t="b">
+        <v>0</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$80.00 </t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N230" t="n">
+        <v>89903939</v>
+      </c>
+      <c r="O230" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>9000000030</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Systems Administrator</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Cobalt Manufacturing is hiring a Systems Administrator to maintain our on-prem and hybrid IT infrastructure across two plants. Responsibilities: administer Windows Server and Active Directory environments; manage backup jobs and patch management schedules; provide escalated support for network and hardware issues; maintain VPN and firewall configurations; support factory-floor systems and industrial network segments. Requirements: 2-4 years of systems administration experience; solid knowledge of Windows Server, Active Directory, and Group Policy; familiarity with networking fundamentals (DNS, DHCP, VPN); comfortable with on-call support rotation.</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Cleveland, OH</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>716</v>
+      </c>
+      <c r="H231" t="b">
+        <v>0</v>
+      </c>
+      <c r="I231" t="n">
+        <v>2856</v>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K231" t="b">
+        <v>0</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$68,000.00 </t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>89903934</v>
+      </c>
+      <c r="O231" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>9000000031</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>IT Systems Administrator</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Anchorline Logistics is looking for an IT Systems Administrator to support a hybrid fleet of Linux and Windows servers for our logistics platform. What You'll Do: manage server provisioning, patching, and monitoring across on-prem and AWS environments; administer Office 365 and identity/access management (Azure AD); maintain backup and disaster recovery procedures; troubleshoot escalated tickets from the helpdesk team. What We Look For: 3+ years of systems administration experience across Linux and Windows; experience with Office 365 / Azure AD administration; solid scripting skills in PowerShell or Bash; strong troubleshooting and documentation habits.</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>809</v>
+      </c>
+      <c r="H232" t="b">
+        <v>1</v>
+      </c>
+      <c r="I232" t="n">
+        <v>658</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K232" t="b">
+        <v>1</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$82,000.00 </t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N232" t="n">
+        <v>89903935</v>
+      </c>
+      <c r="O232" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>9000000032</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Senior Systems Administrator</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Meridian Group is hiring a Senior Systems Administrator to lead infrastructure operations for our corporate office and remote workforce. Responsibilities: own the server, storage, and virtualization environment (VMware); lead patch management and vulnerability remediation efforts with the security team; mentor junior IT staff and review their change requests; manage vendor relationships for hardware and software licensing; plan and execute infrastructure upgrades with minimal downtime. Requirements: 5+ years of systems administration experience; strong VMware and Windows/Linux server administration skills; experience leading infrastructure projects; excellent documentation and communication skills.</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA</t>
+        </is>
+      </c>
+      <c r="G233" t="n">
+        <v>47</v>
+      </c>
+      <c r="H233" t="b">
+        <v>0</v>
+      </c>
+      <c r="I233" t="n">
+        <v>2784</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K233" t="b">
+        <v>0</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$95,000.00 </t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N233" t="n">
+        <v>89903933</v>
+      </c>
+      <c r="O233" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>9000000033</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Linux Systems Administrator</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Vertex Cloud Solutions is seeking a Linux Systems Administrator to support our production and staging server fleet. What You'll Do: manage and patch Linux servers (Ubuntu, RHEL) across cloud and on-prem environments; automate routine administration tasks with Ansible and Bash; monitor system health with Nagios/Prometheus and respond to alerts; support engineering teams with environment provisioning and access requests. What We're Looking For: 2+ years of Linux systems administration experience; solid shell scripting and Ansible or similar automation tooling; understanding of networking and security fundamentals; comfortable working in a fast-paced, cloud-native environment.</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>82</v>
+      </c>
+      <c r="H234" t="b">
+        <v>1</v>
+      </c>
+      <c r="I234" t="n">
+        <v>1928</v>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K234" t="b">
+        <v>0</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$85,000.00 </t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N234" t="n">
+        <v>89903937</v>
+      </c>
+      <c r="O234" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>9000000034</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Junior Systems Administrator</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Harborview Retail is hiring a Junior Systems Administrator to support our IT helpdesk and server operations. Responsibilities: assist with server patching, backups, and user account administration under senior guidance; respond to escalated helpdesk tickets involving hardware, network, or software issues; help maintain documentation for standard IT procedures; support onboarding/offboarding of employee IT equipment and accounts. Requirements: 0-2 years of IT support or systems administration experience; basic knowledge of Windows Server, Active Directory, and networking concepts; strong customer service and troubleshooting mindset; relevant certifications (CompTIA A+/Network+) are a plus.</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>595</v>
+      </c>
+      <c r="H235" t="b">
+        <v>0</v>
+      </c>
+      <c r="I235" t="n">
+        <v>2777</v>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K235" t="b">
+        <v>1</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$55,000.00 </t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N235" t="n">
+        <v>89903929</v>
+      </c>
+      <c r="O235" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>9000000035</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Systems Administrator, Network Operations</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Loopline Commerce is looking for a Systems Administrator to join our network operations team supporting global office connectivity and internal infrastructure. What You'll Do: administer switches, firewalls, and VPN concentrators across office locations; manage internal DNS, DHCP, and monitoring systems; support Zoom Rooms and internal collaboration tooling; participate in an on-call rotation for network incidents. What We Look For: 3+ years of network/systems administration experience; solid understanding of routing, switching, and firewall configuration; experience with monitoring tools (SolarWinds, Nagios, or similar); strong incident response and documentation habits.</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G236" t="n">
+        <v>526</v>
+      </c>
+      <c r="H236" t="b">
+        <v>1</v>
+      </c>
+      <c r="I236" t="n">
+        <v>3441</v>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K236" t="b">
+        <v>0</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$90,000.00 </t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N236" t="n">
+        <v>89903927</v>
+      </c>
+      <c r="O236" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>9000000036</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Nova Consumer Group is hiring a Data Scientist to build models that power personalized recommendations and churn prediction. Responsibilities: design and validate machine learning models using scikit-learn and XGBoost; run A/B tests and analyze statistical significance of product experiments; build feature pipelines from our data warehouse in SQL and Python; communicate findings and model performance to product and marketing stakeholders; collaborate with data engineers on model deployment. Requirements: 3+ years of data science experience; strong Python (pandas, scikit-learn) and SQL skills; solid grounding in statistics and experiment design; experience communicating analytical results to non-technical stakeholders.</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G237" t="n">
+        <v>673</v>
+      </c>
+      <c r="H237" t="b">
+        <v>1</v>
+      </c>
+      <c r="I237" t="n">
+        <v>3958</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K237" t="b">
+        <v>1</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$130,000.00 </t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N237" t="n">
+        <v>89903928</v>
+      </c>
+      <c r="O237" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>9000000037</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Data Scientist, Product Analytics</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Loopline Commerce is seeking a Data Scientist for our Product Analytics team. What You'll Do: design and analyze product experiments to guide roadmap decisions; build predictive models for customer lifetime value and churn; partner with product managers to define success metrics for new features; build self-serve dashboards in Looker for product teams; present quarterly deep-dive analyses to leadership. What We're Looking For: 4+ years of data science or analytics experience in a product-led company; strong SQL and Python skills with experience in scikit-learn or similar; solid understanding of causal inference and experimentation methodology; strong storytelling with data.</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="G238" t="n">
+        <v>157</v>
+      </c>
+      <c r="H238" t="b">
+        <v>1</v>
+      </c>
+      <c r="I238" t="n">
+        <v>2220</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K238" t="b">
+        <v>0</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$145,000.00 </t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N238" t="n">
+        <v>89903927</v>
+      </c>
+      <c r="O238" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>9000000038</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Vertex Cloud Solutions is hiring a Senior Data Scientist to lead modeling initiatives for our SaaS platform's usage-based pricing and forecasting. Responsibilities: design and own forecasting models for customer usage and revenue; lead experimentation strategy across product teams; mentor junior data scientists and review analytical work; partner with engineering on productionizing models via APIs; present strategic recommendations to executive stakeholders. Requirements: 6+ years of data science experience with a track record of shipping models to production; expert-level Python and SQL; strong background in statistical modeling and time-series forecasting; excellent communication and mentorship skills.</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+      <c r="G239" t="n">
+        <v>566</v>
+      </c>
+      <c r="H239" t="b">
+        <v>1</v>
+      </c>
+      <c r="I239" t="n">
+        <v>2352</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K239" t="b">
+        <v>0</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$160,000.00 </t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N239" t="n">
+        <v>89903937</v>
+      </c>
+      <c r="O239" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>9000000039</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Data Scientist, Marketing Analytics</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Brightpath Media is looking for a Data Scientist to support marketing measurement across our client accounts. What You'll Do: build attribution and media mix models to quantify channel performance; analyze campaign data in Python/SQL and present findings to account teams; build reusable dashboards for recurring client reporting; support forecasting of campaign performance for new client pitches. What We Look For: 2+ years of data science or marketing analytics experience; solid Python and SQL skills; familiarity with marketing mix modeling or attribution concepts is a plus; strong communication skills for client-facing analysis.</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G240" t="n">
+        <v>453</v>
+      </c>
+      <c r="H240" t="b">
+        <v>1</v>
+      </c>
+      <c r="I240" t="n">
+        <v>4980</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K240" t="b">
+        <v>0</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$105,000.00 </t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="N240" t="n">
+        <v>89903926</v>
+      </c>
+      <c r="O240" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>9000000040</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Data Scientist, Risk Analytics</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Ledger Financial Systems is hiring a Data Scientist for our Risk Analytics team. Responsibilities: build fraud detection and credit risk models using Python and gradient boosting frameworks; validate model performance against regulatory and fairness requirements; collaborate with engineering to deploy models into real-time transaction scoring; present model governance documentation to internal audit and compliance. Requirements: 4+ years of data science experience, ideally in fintech or risk modeling; strong Python (scikit-learn, XGBoost) and SQL skills; understanding of model validation and fairness/bias considerations; comfortable working in a regulated environment.</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="G241" t="n">
+        <v>239</v>
+      </c>
+      <c r="H241" t="b">
+        <v>0</v>
+      </c>
+      <c r="I241" t="n">
+        <v>1333</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K241" t="b">
+        <v>0</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$150,000.00 </t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N241" t="n">
+        <v>89903936</v>
+      </c>
+      <c r="O241" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>9000000041</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Junior Data Scientist</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Anchorline Logistics is hiring a Junior Data Scientist to support route optimization and demand forecasting analytics. Responsibilities: build and validate forecasting models under senior guidance using Python (pandas, scikit-learn); clean and prepare shipment and warehouse datasets for analysis; build visualizations to communicate findings to operations managers; support ad hoc analysis requests from the operations team. Requirements: 0-2 years of data science experience (internships and academic projects count); strong Python and SQL fundamentals; coursework or project experience with regression, classification, or forecasting; eagerness to learn from senior data scientists.</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G242" t="n">
+        <v>108</v>
+      </c>
+      <c r="H242" t="b">
+        <v>1</v>
+      </c>
+      <c r="I242" t="n">
+        <v>585</v>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K242" t="b">
+        <v>0</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$78,000.00 </t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="N242" t="n">
+        <v>89903935</v>
+      </c>
+      <c r="O242" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>9000000042</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>iOS Developer</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Nova Consumer Group is hiring an iOS Developer to build features for our consumer mobile app used by over a million customers. Responsibilities: build and maintain features in Swift and SwiftUI; work closely with design on pixel-perfect, accessible UI; integrate with backend REST APIs and manage local caching/offline support; write unit and UI tests to keep the app stable across releases; participate in App Store release management. Requirements: 3+ years of iOS development experience; strong Swift and SwiftUI (or UIKit) skills; experience with REST API integration and async/await patterns; familiarity with App Store submission and release processes.</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G243" t="n">
+        <v>171</v>
+      </c>
+      <c r="H243" t="b">
+        <v>1</v>
+      </c>
+      <c r="I243" t="n">
+        <v>5340</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K243" t="b">
+        <v>1</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$125,000.00 </t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N243" t="n">
+        <v>89903928</v>
+      </c>
+      <c r="O243" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>9000000043</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Android Developer</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Loopline Commerce is looking for an Android Developer to build and maintain our shopping app used across millions of devices. What You'll Do: develop features in Kotlin using Jetpack Compose; optimize app performance and startup time across a range of Android devices; integrate push notifications and deep linking for marketing campaigns; write instrumented and unit tests to prevent regressions; collaborate with backend engineers on API contracts. What We're Looking For: 3+ years of Android development experience; strong Kotlin and Jetpack Compose (or XML views) skills; experience with Play Store release processes and staged rollouts; solid understanding of Android app architecture (MVVM).</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="G244" t="n">
+        <v>711</v>
+      </c>
+      <c r="H244" t="b">
+        <v>1</v>
+      </c>
+      <c r="I244" t="n">
+        <v>3658</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K244" t="b">
+        <v>0</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$120,000.00 </t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="N244" t="n">
+        <v>89903927</v>
+      </c>
+      <c r="O244" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>9000000044</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Product Manager, Growth</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Loopline Commerce is hiring a Product Manager to own our growth and activation experience. Responsibilities: define and prioritize a roadmap for onboarding and activation features; partner with engineering and design on discovery and delivery of new experiments; define success metrics and analyze A/B test results with the data team; write clear product specs and manage sprint planning with engineering; present roadmap updates to leadership. Requirements: 4+ years of product management experience, ideally in growth or consumer products; strong analytical skills and comfort with SQL/experiment design; excellent written and verbal communication; experience shipping features end-to-end with cross-functional teams.</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G245" t="n">
+        <v>409</v>
+      </c>
+      <c r="H245" t="b">
+        <v>1</v>
+      </c>
+      <c r="I245" t="n">
+        <v>3326</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K245" t="b">
+        <v>0</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$140,000.00 </t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>Product Management</t>
+        </is>
+      </c>
+      <c r="N245" t="n">
+        <v>89903927</v>
+      </c>
+      <c r="O245" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>9000000045</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Nova Consumer Group is hiring an Associate Product Manager to support our mobile app product team. Responsibilities: write user stories and acceptance criteria for upcoming sprints; conduct competitive research and customer interviews to validate feature ideas; track feature performance in analytics dashboards after launch; coordinate release notes and cross-functional communication for launches; support the senior PM in roadmap planning sessions. Requirements: 0-2 years of product management or related experience (APM programs, consulting, or engineering backgrounds welcome); strong written communication and organizational skills; basic familiarity with analytics tools like Amplitude or Mixpanel; genuine curiosity about user behavior.</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="G246" t="n">
+        <v>494</v>
+      </c>
+      <c r="H246" t="b">
+        <v>0</v>
+      </c>
+      <c r="I246" t="n">
+        <v>4534</v>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="K246" t="b">
+        <v>0</v>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$95,000.00 </t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>Product Management</t>
+        </is>
+      </c>
+      <c r="N246" t="n">
+        <v>89903928</v>
+      </c>
+      <c r="O246" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>9000000046</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Customer Success Specialist</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Brightpath Media is hiring a Customer Success Specialist to support our roster of small business clients. Responsibilities: onboard new clients and guide them through initial campaign setup; respond to client questions via email and chat within SLA; monitor account health metrics and flag at-risk accounts to the account management team; maintain documentation in our knowledge base; gather client feedback to inform product and service improvements. Requirements: 1-3 years in customer success, support, or account management; excellent written communication and empathy for client needs; comfortable using a CRM/helpdesk tool (HubSpot, Zendesk, or similar); organized and able to manage a portfolio of accounts.</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="G247" t="n">
+        <v>581</v>
+      </c>
+      <c r="H247" t="b">
+        <v>1</v>
+      </c>
+      <c r="I247" t="n">
+        <v>294</v>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="K247" t="b">
+        <v>0</v>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$58,000.00 </t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>Customer Success</t>
+        </is>
+      </c>
+      <c r="N247" t="n">
+        <v>89903926</v>
+      </c>
+      <c r="O247" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>9000000047</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Customer Success Manager, SMB</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Harborview Retail is seeking a Customer Success Manager to own retention and growth for our small-to-medium business customer segment. What You'll Do: manage a book of ~150 accounts, driving adoption, renewals, and upsell; run quarterly business reviews with key accounts; partner with product on feature requests surfaced by customers; build playbooks for common onboarding and expansion scenarios; track and report on churn and net revenue retention. What We're Looking For: 3+ years in customer success or account management, ideally in SaaS; strong relationship-building and negotiation skills; comfortable analyzing usage data to identify expansion or churn risk; experience with a CRM such as Salesforce or HubSpot.</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>YEARLY</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="G248" t="n">
+        <v>132</v>
+      </c>
+      <c r="H248" t="b">
+        <v>1</v>
+      </c>
+      <c r="I248" t="n">
+        <v>5784</v>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="K248" t="b">
+        <v>0</v>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$78,000.00 </t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>Customer Success</t>
+        </is>
+      </c>
+      <c r="N248" t="n">
+        <v>89903929</v>
+      </c>
+      <c r="O248" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>